<commit_message>
Address 2nd reviewer claims: S08-S10 descriptive-only flags in T3 (Retail_markets_n/Reporting_status), T9 retitle 'other aquatic products', Fisher exact + G-test sparse fallback (T15), Shapiro-Wilk screening table T18, run_analysis NOTE pointer, docs/drafts updated (Jahan et al. 2024 cited, 2025 hilsa price trend, caveats)
</commit_message>
<xml_diff>
--- a/analysis_outputs/Analysis_Summary.xlsx
+++ b/analysis_outputs/Analysis_Summary.xlsx
@@ -28,6 +28,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T15_Payment_Actor_ChiSquare" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T16_Stratum_Margin_MannWhitney" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T17_Retailer_MC_Profit_Spearman" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T18_ShapiroWilk_Screening" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -496,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E24"/>
+  <dimension ref="B2:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -610,7 +611,7 @@
         <v>11</v>
       </c>
       <c r="E8" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -711,7 +712,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Table 9. Other fish/items purchased by consumers</t>
+          <t>Table 9. Other aquatic products purchased by consumers</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -898,6 +899,24 @@
         <v>31</v>
       </c>
       <c r="E24" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>T18_ShapiroWilk_Screening</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Table 18. Shapiro-Wilk normality screening</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1258,14 +1277,14 @@
     <row r="2">
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Table 9. Other fish/items purchased by consumers</t>
+          <t>Table 9. Other aquatic products purchased by consumers</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Non-focal marine items consumers reported buying (Consumer_Other_Fish sheet).</t>
+          <t>Non-focal aquatic items consumers reported buying on the interview day (Consumer_Other_Fish sheet). Includes crustaceans (Bagda shrimp, Kakra crab) and finfish (Khoira, Datina, Moid, Faisya, lobster) - comparison items outside the ten focal marine-finfish species of Table 3.4.</t>
         </is>
       </c>
     </row>
@@ -6467,7 +6486,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Payment-mode adoption by trader class (Methodology 3.8 Q4). Chi-square on MFS-use frequency (Regular/Occasional/Never); where expected cell counts &lt; 5 the likelihood-ratio (G) test is reported alongside Pearson chi-square as the sparse-cell fallback. Consumer payment method is a separate question and appears in Tables 5/8.</t>
+          <t>Payment-mode adoption by trader class (Methodology 3.8 Q4). Chi-square on MFS-use frequency (Regular/Occasional/Never); because the smallest expected cell &lt; 5, sparse-cell fallbacks are reported alongside Pearson chi-square: the likelihood-ratio (G) test and the exact Freeman-Halton/Fisher test (p from the marginal-conditional enumeration). Consumer payment method is a separate question and appears in Tables 5/8.</t>
         </is>
       </c>
     </row>
@@ -6583,7 +6602,7 @@
       <c r="F8" s="7" t="inlineStr"/>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>chi2=1.22, df=4, p=0.8749, G-test p=0.8809</t>
+          <t>chi2=1.22, df=4, p=0.8749, G-test p=0.8809, Fisher-exact p=0.8945</t>
         </is>
       </c>
     </row>
@@ -7760,6 +7779,166 @@
       </c>
       <c r="F35" s="15" t="n">
         <v>0.0177</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Table 18. Shapiro-Wilk normality screening</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Shapiro-Wilk screening on pooled price series run BEFORE any inferential test, as pre-registered in Methodology 3.8 ('confirmed here by Shapiro-Wilk screening on the pooled series before any test is applied'). Screening motivates the distribution-free battery (Kruskal-Wallis/Mann-Whitney/Wilcoxon) used in Tables 12b/14/16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Series</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>p_value</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Producer price - landing markets M1/M6 (Form A buy)</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>47</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <v>0.8544</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>p&lt;=0.05 - non-normal; nonparametric tests used</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Aratdar auction sell - M1/M6</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>47</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>0.8457</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>p&lt;=0.05 - non-normal; nonparametric tests used</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bepari/Faria sell - all markets</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>135</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>0.9076</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>p&lt;=0.05 - non-normal; nonparametric tests used</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Khuchra retailer sell quotes - all markets</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>128</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>0.8967000000000001</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>p&lt;=0.05 - non-normal; nonparametric tests used</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Consumer-paid prices (Form C slips)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>52</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>p&lt;=0.05 - non-normal; nonparametric tests used</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8728,23 +8907,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:O15"/>
+  <dimension ref="B2:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.6" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="39" customWidth="1" min="4" max="4"/>
     <col width="13.55" customWidth="1" min="5" max="5"/>
-    <col width="17.75" customWidth="1" min="6" max="6"/>
-    <col width="21.95" customWidth="1" min="7" max="7"/>
-    <col width="20.9" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="24.05" customWidth="1" min="11" max="11"/>
+    <col width="18.8" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="17.75" customWidth="1" min="8" max="8"/>
+    <col width="21.95" customWidth="1" min="9" max="9"/>
+    <col width="20.9" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="25.1" customWidth="1" min="13" max="13"/>
-    <col width="21.95" customWidth="1" min="14" max="14"/>
-    <col width="20.9" customWidth="1" min="15" max="15"/>
+    <col width="24.05" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="25.1" customWidth="1" min="15" max="15"/>
+    <col width="21.95" customWidth="1" min="16" max="16"/>
+    <col width="20.9" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -8757,7 +8938,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Producer price = net auction price paid to fishers (Form A buy) at the landing-linked markets M1/M6 only; Aratdar sell = auction hammer price at M1/M6; Bepari sell = Form B sell over all markets; Retailer sell = Form R vendor quote (descriptive; margins use the consumer-paid anchor); Consumer = focal-species purchases actually paid (Form C). Margins = differences of consecutive level means and telescope to the total spread. K/D-flagged prices excluded. Species without a complete chain show blank margins and are excluded from ALL (see Local_name note).</t>
+          <t>Producer price = net auction price paid to fishers (Form A buy) at the landing-linked markets M1/M6 only; Aratdar sell = auction hammer price at M1/M6; Bepari sell = Form B sell over all markets; Retailer sell = Form R vendor quote (descriptive; margins use the consumer-paid anchor); Consumer = focal-species purchases actually paid (Form C). Margins = differences of consecutive level means and telescope to the total spread. K/D-flagged prices excluded. Species without a complete chain show blank margins and are excluded from ALL (see Local_name note). Reporting_status marks species observed in fewer than three markets as descriptive-only (Methodology 3.8): S08/S09/S10 quotes are few and their share figures are indicative, not inferential.</t>
         </is>
       </c>
     </row>
@@ -8784,50 +8965,60 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
+          <t>Retail_markets_n</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Reporting_status</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
           <t>Producer_BDT_kg</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Aratdar_sell_BDT_kg</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Bepari_sell_BDT_kg</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Retailer_sell_BDT_kg</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>Consumer_paid_BDT_kg</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Aratdar_margin_BDT_kg</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Bepari_margin_BDT_kg</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>Retailer_margin_BDT_kg</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>Total_spread_BDT_kg</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="Q4" s="5" t="inlineStr">
         <is>
           <t>Producer_share_pct</t>
         </is>
@@ -8853,33 +9044,36 @@
         <v>71</v>
       </c>
       <c r="F5" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" s="6" t="n">
         <v>1031.62</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="I5" s="6" t="n">
         <v>1083.3</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="J5" s="6" t="n">
         <v>1236.41</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="K5" s="6" t="n">
         <v>1486.96</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="L5" s="6" t="n">
         <v>1420</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="M5" s="6" t="n">
         <v>51.68</v>
       </c>
-      <c r="L5" s="6" t="n">
+      <c r="N5" s="6" t="n">
         <v>153.11</v>
       </c>
-      <c r="M5" s="6" t="n">
+      <c r="O5" s="6" t="n">
         <v>183.59</v>
       </c>
-      <c r="N5" s="6" t="n">
+      <c r="P5" s="6" t="n">
         <v>388.38</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="Q5" s="6" t="n">
         <v>72.59999999999999</v>
       </c>
     </row>
@@ -8903,33 +9097,37 @@
         <v>64</v>
       </c>
       <c r="F6" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="8" t="n">
         <v>1110.67</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="I6" s="8" t="n">
         <v>1165.59</v>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="J6" s="8" t="n">
         <v>1378.04</v>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="K6" s="8" t="n">
         <v>1619.16</v>
       </c>
-      <c r="J6" s="8" t="n">
+      <c r="L6" s="8" t="n">
         <v>1615</v>
       </c>
-      <c r="K6" s="8" t="n">
+      <c r="M6" s="8" t="n">
         <v>54.92</v>
       </c>
-      <c r="L6" s="8" t="n">
+      <c r="N6" s="8" t="n">
         <v>212.45</v>
       </c>
-      <c r="M6" s="8" t="n">
+      <c r="O6" s="8" t="n">
         <v>236.96</v>
       </c>
-      <c r="N6" s="8" t="n">
+      <c r="P6" s="8" t="n">
         <v>504.33</v>
       </c>
-      <c r="O6" s="8" t="n">
+      <c r="Q6" s="8" t="n">
         <v>68.8</v>
       </c>
     </row>
@@ -8953,33 +9151,36 @@
         <v>52</v>
       </c>
       <c r="F7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="6" t="n">
         <v>735.53</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="I7" s="6" t="n">
         <v>771.7</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="J7" s="6" t="n">
         <v>886.61</v>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="K7" s="6" t="n">
         <v>1069.64</v>
       </c>
-      <c r="J7" s="6" t="n">
+      <c r="L7" s="6" t="n">
         <v>1033.33</v>
       </c>
-      <c r="K7" s="6" t="n">
+      <c r="M7" s="6" t="n">
         <v>36.17</v>
       </c>
-      <c r="L7" s="6" t="n">
+      <c r="N7" s="6" t="n">
         <v>114.91</v>
       </c>
-      <c r="M7" s="6" t="n">
+      <c r="O7" s="6" t="n">
         <v>146.72</v>
       </c>
-      <c r="N7" s="6" t="n">
+      <c r="P7" s="6" t="n">
         <v>297.8</v>
       </c>
-      <c r="O7" s="6" t="n">
+      <c r="Q7" s="6" t="n">
         <v>71.2</v>
       </c>
     </row>
@@ -9003,33 +9204,37 @@
         <v>46</v>
       </c>
       <c r="F8" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" s="7" t="inlineStr"/>
+      <c r="H8" s="8" t="n">
         <v>660.95</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="I8" s="8" t="n">
         <v>687.75</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="J8" s="8" t="n">
         <v>762.77</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="K8" s="8" t="n">
         <v>933.4400000000001</v>
       </c>
-      <c r="J8" s="8" t="n">
+      <c r="L8" s="8" t="n">
         <v>885</v>
       </c>
-      <c r="K8" s="8" t="n">
+      <c r="M8" s="8" t="n">
         <v>26.8</v>
       </c>
-      <c r="L8" s="8" t="n">
+      <c r="N8" s="8" t="n">
         <v>75.02</v>
       </c>
-      <c r="M8" s="8" t="n">
+      <c r="O8" s="8" t="n">
         <v>122.23</v>
       </c>
-      <c r="N8" s="8" t="n">
+      <c r="P8" s="8" t="n">
         <v>224.05</v>
       </c>
-      <c r="O8" s="8" t="n">
+      <c r="Q8" s="8" t="n">
         <v>74.7</v>
       </c>
     </row>
@@ -9053,33 +9258,36 @@
         <v>74</v>
       </c>
       <c r="F9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" s="6" t="n">
         <v>407.79</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="I9" s="6" t="n">
         <v>428.72</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="J9" s="6" t="n">
         <v>501.77</v>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="K9" s="6" t="n">
         <v>581.23</v>
       </c>
-      <c r="J9" s="6" t="n">
+      <c r="L9" s="6" t="n">
         <v>585</v>
       </c>
-      <c r="K9" s="6" t="n">
+      <c r="M9" s="6" t="n">
         <v>20.93</v>
       </c>
-      <c r="L9" s="6" t="n">
+      <c r="N9" s="6" t="n">
         <v>73.05</v>
       </c>
-      <c r="M9" s="6" t="n">
+      <c r="O9" s="6" t="n">
         <v>83.23</v>
       </c>
-      <c r="N9" s="6" t="n">
+      <c r="P9" s="6" t="n">
         <v>177.21</v>
       </c>
-      <c r="O9" s="6" t="n">
+      <c r="Q9" s="6" t="n">
         <v>69.7</v>
       </c>
     </row>
@@ -9103,33 +9311,37 @@
         <v>63</v>
       </c>
       <c r="F10" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G10" s="7" t="inlineStr"/>
+      <c r="H10" s="8" t="n">
         <v>314.1</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="I10" s="8" t="n">
         <v>323.55</v>
       </c>
-      <c r="H10" s="8" t="n">
+      <c r="J10" s="8" t="n">
         <v>380.42</v>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="K10" s="8" t="n">
         <v>457.13</v>
       </c>
-      <c r="J10" s="8" t="n">
+      <c r="L10" s="8" t="n">
         <v>446.54</v>
       </c>
-      <c r="K10" s="8" t="n">
+      <c r="M10" s="8" t="n">
         <v>9.449999999999999</v>
       </c>
-      <c r="L10" s="8" t="n">
+      <c r="N10" s="8" t="n">
         <v>56.87</v>
       </c>
-      <c r="M10" s="8" t="n">
+      <c r="O10" s="8" t="n">
         <v>66.12</v>
       </c>
-      <c r="N10" s="8" t="n">
+      <c r="P10" s="8" t="n">
         <v>132.44</v>
       </c>
-      <c r="O10" s="8" t="n">
+      <c r="Q10" s="8" t="n">
         <v>70.3</v>
       </c>
     </row>
@@ -9153,33 +9365,36 @@
         <v>29</v>
       </c>
       <c r="F11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" s="6" t="n">
         <v>361.74</v>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="I11" s="6" t="n">
         <v>377.81</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="J11" s="6" t="n">
         <v>450.16</v>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="K11" s="6" t="n">
         <v>545.45</v>
       </c>
-      <c r="J11" s="6" t="n">
+      <c r="L11" s="6" t="n">
         <v>530</v>
       </c>
-      <c r="K11" s="6" t="n">
+      <c r="M11" s="6" t="n">
         <v>16.07</v>
       </c>
-      <c r="L11" s="6" t="n">
+      <c r="N11" s="6" t="n">
         <v>72.34999999999999</v>
       </c>
-      <c r="M11" s="6" t="n">
+      <c r="O11" s="6" t="n">
         <v>79.84</v>
       </c>
-      <c r="N11" s="6" t="n">
+      <c r="P11" s="6" t="n">
         <v>168.26</v>
       </c>
-      <c r="O11" s="6" t="n">
+      <c r="Q11" s="6" t="n">
         <v>68.3</v>
       </c>
     </row>
@@ -9203,33 +9418,41 @@
         <v>9</v>
       </c>
       <c r="F12" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Descriptive-only (Method 3.8)</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="n">
         <v>231.78</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="I12" s="8" t="n">
         <v>241.16</v>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="J12" s="8" t="n">
         <v>279.01</v>
       </c>
-      <c r="I12" s="8" t="n">
+      <c r="K12" s="8" t="n">
         <v>325</v>
       </c>
-      <c r="J12" s="8" t="n">
+      <c r="L12" s="8" t="n">
         <v>330</v>
       </c>
-      <c r="K12" s="8" t="n">
+      <c r="M12" s="8" t="n">
         <v>9.380000000000001</v>
       </c>
-      <c r="L12" s="8" t="n">
+      <c r="N12" s="8" t="n">
         <v>37.85</v>
       </c>
-      <c r="M12" s="8" t="n">
+      <c r="O12" s="8" t="n">
         <v>50.99</v>
       </c>
-      <c r="N12" s="8" t="n">
+      <c r="P12" s="8" t="n">
         <v>98.22</v>
       </c>
-      <c r="O12" s="8" t="n">
+      <c r="Q12" s="8" t="n">
         <v>70.2</v>
       </c>
     </row>
@@ -9253,33 +9476,41 @@
         <v>15</v>
       </c>
       <c r="F13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Descriptive-only (Method 3.8)</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n">
         <v>188.91</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="I13" s="6" t="n">
         <v>195.61</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="J13" s="6" t="n">
         <v>234.46</v>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="K13" s="6" t="n">
         <v>263.01</v>
       </c>
-      <c r="J13" s="6" t="n">
+      <c r="L13" s="6" t="n">
         <v>267.5</v>
       </c>
-      <c r="K13" s="6" t="n">
+      <c r="M13" s="6" t="n">
         <v>6.7</v>
       </c>
-      <c r="L13" s="6" t="n">
+      <c r="N13" s="6" t="n">
         <v>38.85</v>
       </c>
-      <c r="M13" s="6" t="n">
+      <c r="O13" s="6" t="n">
         <v>33.04</v>
       </c>
-      <c r="N13" s="6" t="n">
+      <c r="P13" s="6" t="n">
         <v>78.59</v>
       </c>
-      <c r="O13" s="6" t="n">
+      <c r="Q13" s="6" t="n">
         <v>70.59999999999999</v>
       </c>
     </row>
@@ -9303,23 +9534,31 @@
         <v>6</v>
       </c>
       <c r="F14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Descriptive-only (Method 3.8)</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="n">
         <v>163.45</v>
       </c>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="8" t="n">
+      <c r="I14" s="7" t="n"/>
+      <c r="J14" s="8" t="n">
         <v>179.53</v>
       </c>
-      <c r="I14" s="8" t="n">
+      <c r="K14" s="8" t="n">
         <v>230</v>
       </c>
-      <c r="J14" s="8" t="n">
+      <c r="L14" s="8" t="n">
         <v>215</v>
       </c>
-      <c r="K14" s="7" t="n"/>
-      <c r="L14" s="7" t="n"/>
       <c r="M14" s="7" t="n"/>
       <c r="N14" s="7" t="n"/>
-      <c r="O14" s="8" t="n">
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" s="7" t="n"/>
+      <c r="Q14" s="8" t="n">
         <v>76</v>
       </c>
     </row>
@@ -9342,34 +9581,39 @@
       <c r="E15" t="n">
         <v>423</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Pooled over chain-complete species</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="n">
         <v>560.34</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="I15" s="6" t="n">
         <v>586.13</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="J15" s="6" t="n">
         <v>678.85</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="K15" s="6" t="n">
         <v>809</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="L15" s="6" t="n">
         <v>790.26</v>
       </c>
-      <c r="K15" s="6" t="n">
+      <c r="M15" s="6" t="n">
         <v>25.79</v>
       </c>
-      <c r="L15" s="6" t="n">
+      <c r="N15" s="6" t="n">
         <v>92.72</v>
       </c>
-      <c r="M15" s="6" t="n">
+      <c r="O15" s="6" t="n">
         <v>111.41</v>
       </c>
-      <c r="N15" s="6" t="n">
+      <c r="P15" s="6" t="n">
         <v>229.92</v>
       </c>
-      <c r="O15" s="6" t="n">
+      <c r="Q15" s="6" t="n">
         <v>70.90000000000001</v>
       </c>
     </row>
@@ -10377,14 +10621,14 @@
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Supply syndicate control</t>
+          <t>Unsold fish spoilage loss</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>36.7</v>
+        <v>40</v>
       </c>
       <c r="E5" t="n">
         <v>9</v>
@@ -10393,10 +10637,10 @@
         <v>30</v>
       </c>
       <c r="G5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>26.7</v>
+        <v>23.3</v>
       </c>
       <c r="I5" t="n">
         <v>28</v>
@@ -10408,14 +10652,14 @@
     <row r="6">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Unsold fish spoilage loss</t>
+          <t>Supply syndicate control</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>40</v>
+        <v>36.7</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>9</v>
@@ -10424,10 +10668,10 @@
         <v>30</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>23.3</v>
+        <v>26.7</v>
       </c>
       <c r="I6" s="7" t="n">
         <v>28</v>
@@ -10532,26 +10776,26 @@
     <row r="10">
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Waterlogging during monsoon</t>
+          <t>Low landings in lean season</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>23.3</v>
+        <v>30</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>20</v>
+        <v>26.7</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>30</v>
+        <v>16.7</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>22</v>
@@ -10563,26 +10807,26 @@
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>Low landings in lean season</t>
+          <t>Waterlogging during monsoon</t>
         </is>
       </c>
       <c r="C11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>6</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="G11" t="n">
         <v>9</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="H11" s="6" t="n">
         <v>30</v>
-      </c>
-      <c r="E11" t="n">
-        <v>8</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="G11" t="n">
-        <v>5</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>16.7</v>
       </c>
       <c r="I11" t="n">
         <v>22</v>
@@ -10592,22 +10836,22 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Rising cost of ice and salt</t>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Irregular electricity and load-shedding</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>26.7</v>
+        <v>13.3</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>7</v>
@@ -10623,22 +10867,22 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Irregular electricity and load-shedding</t>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Rising cost of ice and salt</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>13.3</v>
+        <v>26.7</v>
       </c>
       <c r="G13" t="n">
         <v>7</v>

</xml_diff>

<commit_message>
Post-merge consistency: deterministic tie ordering in T6 problems table (was hash-random set order); regenerate all outputs from merged code
</commit_message>
<xml_diff>
--- a/analysis_outputs/Analysis_Summary.xlsx
+++ b/analysis_outputs/Analysis_Summary.xlsx
@@ -10621,14 +10621,14 @@
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Unsold fish spoilage loss</t>
+          <t>Supply syndicate control</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>40</v>
+        <v>36.7</v>
       </c>
       <c r="E5" t="n">
         <v>9</v>
@@ -10637,10 +10637,10 @@
         <v>30</v>
       </c>
       <c r="G5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>23.3</v>
+        <v>26.7</v>
       </c>
       <c r="I5" t="n">
         <v>28</v>
@@ -10652,14 +10652,14 @@
     <row r="6">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Supply syndicate control</t>
+          <t>Unsold fish spoilage loss</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>36.7</v>
+        <v>40</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>9</v>
@@ -10668,10 +10668,10 @@
         <v>30</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>26.7</v>
+        <v>23.3</v>
       </c>
       <c r="I6" s="7" t="n">
         <v>28</v>
@@ -10900,20 +10900,20 @@
     <row r="14">
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Rising toll and lease burden</t>
+          <t>Delayed credit recovery</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>16.7</v>
+        <v>20</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>26.7</v>
+        <v>23.3</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>7</v>
@@ -10931,20 +10931,20 @@
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>Delayed credit recovery</t>
+          <t>Rising toll and lease burden</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>20</v>
+        <v>16.7</v>
       </c>
       <c r="E15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>23.3</v>
+        <v>26.7</v>
       </c>
       <c r="G15" t="n">
         <v>7</v>

</xml_diff>

<commit_message>
Round-3 review fixes: report producer shares only with >=3 consumer-paid quotes (MIN_CONS); T3 gains Consumer_paid_n column; S08/S10 share cells blanked; ALL/T10 pool = 8 chain-complete species; review_audit aligned to same rule (62/3/0); docs/drafts updated to new margins (27.8/99.6/119.0, spread 246.4)
</commit_message>
<xml_diff>
--- a/analysis_outputs/Analysis_Summary.xlsx
+++ b/analysis_outputs/Analysis_Summary.xlsx
@@ -611,7 +611,7 @@
         <v>11</v>
       </c>
       <c r="E8" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1471,7 +1471,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Unweighted means of species-level means over chain-complete species only (n_species=9; see Table 3 note). Producer &amp; auction prices from landing-linked markets M1/M6 (first-sale proxy, Methodology 3.11c); wholesale price = Bepari sell over all markets; retail price = consumer-paid anchor (Form C slips). Margins are differences of consecutive level means, so they sum exactly to the total spread and PS% + spread% = 100. Margin % is expressed as a share of the pooled consumer price.</t>
+          <t>Unweighted means of species-level means over chain-complete species only (n_species=8; see Table 3 note). Producer &amp; auction prices from landing-linked markets M1/M6 (first-sale proxy, Methodology 3.11c); wholesale price = Bepari sell over all markets; retail price = consumer-paid anchor (Form C slips). Margins are differences of consecutive level means, so they sum exactly to the total spread and PS% + spread% = 100. Margin % is expressed as a share of the pooled consumer price.</t>
         </is>
       </c>
     </row>
@@ -1504,10 +1504,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>25.79</v>
+        <v>27.84</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>3.3</v>
@@ -1520,10 +1520,10 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>92.72</v>
+        <v>99.58</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>11.7</v>
@@ -1536,13 +1536,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>111.41</v>
+        <v>118.97</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>14.1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -1552,10 +1552,10 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>229.92</v>
+        <v>246.39</v>
       </c>
       <c r="E8" s="8" t="n">
         <v>29.1</v>
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>70.90000000000001</v>
@@ -8907,7 +8907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:Q15"/>
+  <dimension ref="B2:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.6" customWidth="1" min="2" max="2"/>
@@ -8915,17 +8915,18 @@
     <col width="39" customWidth="1" min="4" max="4"/>
     <col width="13.55" customWidth="1" min="5" max="5"/>
     <col width="18.8" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="17.75" customWidth="1" min="8" max="8"/>
-    <col width="21.95" customWidth="1" min="9" max="9"/>
-    <col width="20.9" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="17.75" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="17.75" customWidth="1" min="9" max="9"/>
+    <col width="21.95" customWidth="1" min="10" max="10"/>
+    <col width="20.9" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="24.05" customWidth="1" min="13" max="13"/>
-    <col width="23" customWidth="1" min="14" max="14"/>
-    <col width="25.1" customWidth="1" min="15" max="15"/>
-    <col width="21.95" customWidth="1" min="16" max="16"/>
-    <col width="20.9" customWidth="1" min="17" max="17"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="24.05" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="15" max="15"/>
+    <col width="25.1" customWidth="1" min="16" max="16"/>
+    <col width="21.95" customWidth="1" min="17" max="17"/>
+    <col width="20.9" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -8938,7 +8939,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Producer price = net auction price paid to fishers (Form A buy) at the landing-linked markets M1/M6 only; Aratdar sell = auction hammer price at M1/M6; Bepari sell = Form B sell over all markets; Retailer sell = Form R vendor quote (descriptive; margins use the consumer-paid anchor); Consumer = focal-species purchases actually paid (Form C). Margins = differences of consecutive level means and telescope to the total spread. K/D-flagged prices excluded. Species without a complete chain show blank margins and are excluded from ALL (see Local_name note). Reporting_status marks species observed in fewer than three markets as descriptive-only (Methodology 3.8): S08/S09/S10 quotes are few and their share figures are indicative, not inferential.</t>
+          <t>Producer price = net auction price paid to fishers (Form A buy) at the landing-linked markets M1/M6 only; Aratdar sell = auction hammer price at M1/M6; Bepari sell = Form B sell over all markets; Retailer sell = Form R vendor quote (descriptive; margins use the consumer-paid anchor); Consumer = focal-species purchases actually paid (Form C). Margins = differences of consecutive level means and telescope to the total spread. K/D-flagged prices excluded. Species without a complete chain - or with fewer than MIN_CONS consumer-paid observations - show prices but blank margins/share and are excluded from ALL (see Local_name note); Consumer_paid_n reports the actual number of consumer slips behind each share. Reporting_status lists Method 3.8 descriptive-only reasons (S08/S09/S10 in the current set).</t>
         </is>
       </c>
     </row>
@@ -8970,55 +8971,60 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
+          <t>Consumer_paid_n</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
           <t>Reporting_status</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Producer_BDT_kg</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Aratdar_sell_BDT_kg</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Bepari_sell_BDT_kg</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>Retailer_sell_BDT_kg</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Consumer_paid_BDT_kg</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Aratdar_margin_BDT_kg</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>Bepari_margin_BDT_kg</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>Retailer_margin_BDT_kg</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="Q4" s="5" t="inlineStr">
         <is>
           <t>Total_spread_BDT_kg</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="R4" s="5" t="inlineStr">
         <is>
           <t>Producer_share_pct</t>
         </is>
@@ -9046,34 +9052,37 @@
       <c r="F5" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="G5" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>1031.62</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="J5" s="6" t="n">
         <v>1083.3</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="K5" s="6" t="n">
         <v>1236.41</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="L5" s="6" t="n">
         <v>1486.96</v>
       </c>
-      <c r="L5" s="6" t="n">
+      <c r="M5" s="6" t="n">
         <v>1420</v>
       </c>
-      <c r="M5" s="6" t="n">
+      <c r="N5" s="6" t="n">
         <v>51.68</v>
       </c>
-      <c r="N5" s="6" t="n">
+      <c r="O5" s="6" t="n">
         <v>153.11</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="P5" s="6" t="n">
         <v>183.59</v>
       </c>
-      <c r="P5" s="6" t="n">
+      <c r="Q5" s="6" t="n">
         <v>388.38</v>
       </c>
-      <c r="Q5" s="6" t="n">
+      <c r="R5" s="6" t="n">
         <v>72.59999999999999</v>
       </c>
     </row>
@@ -9099,35 +9108,38 @@
       <c r="F6" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="8" t="n">
+      <c r="G6" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" s="7" t="inlineStr"/>
+      <c r="I6" s="8" t="n">
         <v>1110.67</v>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="J6" s="8" t="n">
         <v>1165.59</v>
       </c>
-      <c r="J6" s="8" t="n">
+      <c r="K6" s="8" t="n">
         <v>1378.04</v>
       </c>
-      <c r="K6" s="8" t="n">
+      <c r="L6" s="8" t="n">
         <v>1619.16</v>
       </c>
-      <c r="L6" s="8" t="n">
+      <c r="M6" s="8" t="n">
         <v>1615</v>
       </c>
-      <c r="M6" s="8" t="n">
+      <c r="N6" s="8" t="n">
         <v>54.92</v>
       </c>
-      <c r="N6" s="8" t="n">
+      <c r="O6" s="8" t="n">
         <v>212.45</v>
       </c>
-      <c r="O6" s="8" t="n">
+      <c r="P6" s="8" t="n">
         <v>236.96</v>
       </c>
-      <c r="P6" s="8" t="n">
+      <c r="Q6" s="8" t="n">
         <v>504.33</v>
       </c>
-      <c r="Q6" s="8" t="n">
+      <c r="R6" s="8" t="n">
         <v>68.8</v>
       </c>
     </row>
@@ -9153,34 +9165,37 @@
       <c r="F7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="G7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="6" t="n">
         <v>735.53</v>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="J7" s="6" t="n">
         <v>771.7</v>
       </c>
-      <c r="J7" s="6" t="n">
+      <c r="K7" s="6" t="n">
         <v>886.61</v>
       </c>
-      <c r="K7" s="6" t="n">
+      <c r="L7" s="6" t="n">
         <v>1069.64</v>
       </c>
-      <c r="L7" s="6" t="n">
+      <c r="M7" s="6" t="n">
         <v>1033.33</v>
       </c>
-      <c r="M7" s="6" t="n">
+      <c r="N7" s="6" t="n">
         <v>36.17</v>
       </c>
-      <c r="N7" s="6" t="n">
+      <c r="O7" s="6" t="n">
         <v>114.91</v>
       </c>
-      <c r="O7" s="6" t="n">
+      <c r="P7" s="6" t="n">
         <v>146.72</v>
       </c>
-      <c r="P7" s="6" t="n">
+      <c r="Q7" s="6" t="n">
         <v>297.8</v>
       </c>
-      <c r="Q7" s="6" t="n">
+      <c r="R7" s="6" t="n">
         <v>71.2</v>
       </c>
     </row>
@@ -9206,35 +9221,38 @@
       <c r="F8" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="8" t="n">
+      <c r="G8" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" s="7" t="inlineStr"/>
+      <c r="I8" s="8" t="n">
         <v>660.95</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="J8" s="8" t="n">
         <v>687.75</v>
       </c>
-      <c r="J8" s="8" t="n">
+      <c r="K8" s="8" t="n">
         <v>762.77</v>
       </c>
-      <c r="K8" s="8" t="n">
+      <c r="L8" s="8" t="n">
         <v>933.4400000000001</v>
       </c>
-      <c r="L8" s="8" t="n">
+      <c r="M8" s="8" t="n">
         <v>885</v>
       </c>
-      <c r="M8" s="8" t="n">
+      <c r="N8" s="8" t="n">
         <v>26.8</v>
       </c>
-      <c r="N8" s="8" t="n">
+      <c r="O8" s="8" t="n">
         <v>75.02</v>
       </c>
-      <c r="O8" s="8" t="n">
+      <c r="P8" s="8" t="n">
         <v>122.23</v>
       </c>
-      <c r="P8" s="8" t="n">
+      <c r="Q8" s="8" t="n">
         <v>224.05</v>
       </c>
-      <c r="Q8" s="8" t="n">
+      <c r="R8" s="8" t="n">
         <v>74.7</v>
       </c>
     </row>
@@ -9260,34 +9278,37 @@
       <c r="F9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="G9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I9" s="6" t="n">
         <v>407.79</v>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="J9" s="6" t="n">
         <v>428.72</v>
       </c>
-      <c r="J9" s="6" t="n">
+      <c r="K9" s="6" t="n">
         <v>501.77</v>
       </c>
-      <c r="K9" s="6" t="n">
+      <c r="L9" s="6" t="n">
         <v>581.23</v>
       </c>
-      <c r="L9" s="6" t="n">
+      <c r="M9" s="6" t="n">
         <v>585</v>
       </c>
-      <c r="M9" s="6" t="n">
+      <c r="N9" s="6" t="n">
         <v>20.93</v>
       </c>
-      <c r="N9" s="6" t="n">
+      <c r="O9" s="6" t="n">
         <v>73.05</v>
       </c>
-      <c r="O9" s="6" t="n">
+      <c r="P9" s="6" t="n">
         <v>83.23</v>
       </c>
-      <c r="P9" s="6" t="n">
+      <c r="Q9" s="6" t="n">
         <v>177.21</v>
       </c>
-      <c r="Q9" s="6" t="n">
+      <c r="R9" s="6" t="n">
         <v>69.7</v>
       </c>
     </row>
@@ -9313,35 +9334,38 @@
       <c r="F10" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="8" t="n">
+      <c r="G10" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="H10" s="7" t="inlineStr"/>
+      <c r="I10" s="8" t="n">
         <v>314.1</v>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="J10" s="8" t="n">
         <v>323.55</v>
       </c>
-      <c r="J10" s="8" t="n">
+      <c r="K10" s="8" t="n">
         <v>380.42</v>
       </c>
-      <c r="K10" s="8" t="n">
+      <c r="L10" s="8" t="n">
         <v>457.13</v>
       </c>
-      <c r="L10" s="8" t="n">
+      <c r="M10" s="8" t="n">
         <v>446.54</v>
       </c>
-      <c r="M10" s="8" t="n">
+      <c r="N10" s="8" t="n">
         <v>9.449999999999999</v>
       </c>
-      <c r="N10" s="8" t="n">
+      <c r="O10" s="8" t="n">
         <v>56.87</v>
       </c>
-      <c r="O10" s="8" t="n">
+      <c r="P10" s="8" t="n">
         <v>66.12</v>
       </c>
-      <c r="P10" s="8" t="n">
+      <c r="Q10" s="8" t="n">
         <v>132.44</v>
       </c>
-      <c r="Q10" s="8" t="n">
+      <c r="R10" s="8" t="n">
         <v>70.3</v>
       </c>
     </row>
@@ -9367,34 +9391,37 @@
       <c r="F11" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="G11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="I11" s="6" t="n">
         <v>361.74</v>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="J11" s="6" t="n">
         <v>377.81</v>
       </c>
-      <c r="J11" s="6" t="n">
+      <c r="K11" s="6" t="n">
         <v>450.16</v>
       </c>
-      <c r="K11" s="6" t="n">
+      <c r="L11" s="6" t="n">
         <v>545.45</v>
       </c>
-      <c r="L11" s="6" t="n">
+      <c r="M11" s="6" t="n">
         <v>530</v>
       </c>
-      <c r="M11" s="6" t="n">
+      <c r="N11" s="6" t="n">
         <v>16.07</v>
       </c>
-      <c r="N11" s="6" t="n">
+      <c r="O11" s="6" t="n">
         <v>72.34999999999999</v>
       </c>
-      <c r="O11" s="6" t="n">
+      <c r="P11" s="6" t="n">
         <v>79.84</v>
       </c>
-      <c r="P11" s="6" t="n">
+      <c r="Q11" s="6" t="n">
         <v>168.26</v>
       </c>
-      <c r="Q11" s="6" t="n">
+      <c r="R11" s="6" t="n">
         <v>68.3</v>
       </c>
     </row>
@@ -9420,41 +9447,34 @@
       <c r="F12" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>Descriptive-only (Method 3.8)</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="n">
+      <c r="G12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Descriptive-only (Method 3.8): retail quotes in 2 market(s); consumer quotes n=1 (&lt;3; share not reported)</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="n">
         <v>231.78</v>
       </c>
-      <c r="I12" s="8" t="n">
+      <c r="J12" s="8" t="n">
         <v>241.16</v>
       </c>
-      <c r="J12" s="8" t="n">
+      <c r="K12" s="8" t="n">
         <v>279.01</v>
       </c>
-      <c r="K12" s="8" t="n">
+      <c r="L12" s="8" t="n">
         <v>325</v>
       </c>
-      <c r="L12" s="8" t="n">
+      <c r="M12" s="8" t="n">
         <v>330</v>
       </c>
-      <c r="M12" s="8" t="n">
-        <v>9.380000000000001</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>37.85</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>50.99</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>98.22</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>70.2</v>
-      </c>
+      <c r="N12" s="7" t="n"/>
+      <c r="O12" s="7" t="n"/>
+      <c r="P12" s="7" t="n"/>
+      <c r="Q12" s="7" t="n"/>
+      <c r="R12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
@@ -9478,39 +9498,42 @@
       <c r="F13" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Descriptive-only (Method 3.8)</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="n">
+      <c r="G13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Descriptive-only (Method 3.8): retail quotes in 2 market(s)</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n">
         <v>188.91</v>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="J13" s="6" t="n">
         <v>195.61</v>
       </c>
-      <c r="J13" s="6" t="n">
+      <c r="K13" s="6" t="n">
         <v>234.46</v>
       </c>
-      <c r="K13" s="6" t="n">
+      <c r="L13" s="6" t="n">
         <v>263.01</v>
       </c>
-      <c r="L13" s="6" t="n">
+      <c r="M13" s="6" t="n">
         <v>267.5</v>
       </c>
-      <c r="M13" s="6" t="n">
+      <c r="N13" s="6" t="n">
         <v>6.7</v>
       </c>
-      <c r="N13" s="6" t="n">
+      <c r="O13" s="6" t="n">
         <v>38.85</v>
       </c>
-      <c r="O13" s="6" t="n">
+      <c r="P13" s="6" t="n">
         <v>33.04</v>
       </c>
-      <c r="P13" s="6" t="n">
+      <c r="Q13" s="6" t="n">
         <v>78.59</v>
       </c>
-      <c r="Q13" s="6" t="n">
+      <c r="R13" s="6" t="n">
         <v>70.59999999999999</v>
       </c>
     </row>
@@ -9536,31 +9559,32 @@
       <c r="F14" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Descriptive-only (Method 3.8)</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="n">
+      <c r="G14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Descriptive-only (Method 3.8): retail quotes in 1 market(s); consumer quotes n=1 (&lt;3; share not reported)</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="n">
         <v>163.45</v>
       </c>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="8" t="n">
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="8" t="n">
         <v>179.53</v>
       </c>
-      <c r="K14" s="8" t="n">
+      <c r="L14" s="8" t="n">
         <v>230</v>
       </c>
-      <c r="L14" s="8" t="n">
+      <c r="M14" s="8" t="n">
         <v>215</v>
       </c>
-      <c r="M14" s="7" t="n"/>
       <c r="N14" s="7" t="n"/>
       <c r="O14" s="7" t="n"/>
       <c r="P14" s="7" t="n"/>
-      <c r="Q14" s="8" t="n">
-        <v>76</v>
-      </c>
+      <c r="Q14" s="7" t="n"/>
+      <c r="R14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
@@ -9570,7 +9594,7 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Mean of species means (chain-complete: S01, S02, S03, S04, S05, S06, S07, S08, S09)</t>
+          <t>Mean of species means (chain-complete: S01, S02, S03, S04, S05, S06, S07, S09)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -9579,41 +9603,41 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>423</v>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>Pooled over chain-complete species</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>560.34</v>
+        <v>414</v>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Pooled over 8 chain-complete species (consumer n &gt;= 3)</t>
+        </is>
       </c>
       <c r="I15" s="6" t="n">
-        <v>586.13</v>
+        <v>601.41</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>678.85</v>
+        <v>629.25</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>809</v>
+        <v>728.83</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>790.26</v>
+        <v>869.5</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.79</v>
+        <v>847.8</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>92.72</v>
+        <v>27.84</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>111.41</v>
+        <v>99.58</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>229.92</v>
+        <v>118.97</v>
       </c>
       <c r="Q15" s="6" t="n">
+        <v>246.39</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>70.90000000000001</v>
       </c>
     </row>

</xml_diff>